<commit_message>
refactor: enhance application security with file upload validation, CSRF delete forms, database hardening, and new test suites
</commit_message>
<xml_diff>
--- a/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
+++ b/public/excel/Laporan-Presensi-UKM-ukm-taekwondo.xlsx
@@ -20,7 +20,7 @@
     <t>LAPORAN PRESENSI UKM UKM TAEKWONDO</t>
   </si>
   <si>
-    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 13/09/2026</t>
+    <t>Politeknik Pembangunan Pertanian Malang - Tanggal Cetak: 21/09/2026</t>
   </si>
   <si>
     <t>Rentang Tanggal: - s/d -</t>
@@ -47,13 +47,13 @@
     <t>Status Kehadiran</t>
   </si>
   <si>
-    <t>Bailey Denesik</t>
+    <t>Dave White III</t>
   </si>
   <si>
     <t>Ujian Kenaikan Sabuk</t>
   </si>
   <si>
-    <t>13/09/2026</t>
+    <t>21/09/2026</t>
   </si>
   <si>
     <t>-</t>
@@ -481,7 +481,7 @@
         <v>10</v>
       </c>
       <c r="C6">
-        <v>6222102924</v>
+        <v>8521509148</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>

</xml_diff>